<commit_message>
Verify first outreach prospect contacts
</commit_message>
<xml_diff>
--- a/sales/CyberVSI_90_Day_Client_Pipeline.xlsx
+++ b/sales/CyberVSI_90_Day_Client_Pipeline.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4d7a93b6a13c43bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospect Pipeline" sheetId="2" r:id="Ra407de5a29b04efc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Plan" sheetId="3" r:id="R9af67e6a280b4f7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lean Budget" sheetId="4" r:id="R881e16b44dc04758"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach Drafts" sheetId="5" r:id="R333237b420584502"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R44d873791b7f4da5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospect Pipeline" sheetId="2" r:id="Rf8d1d99a589a4d98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13-Week Plan" sheetId="3" r:id="Radb0f77f25ce4f20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lean Budget" sheetId="4" r:id="R3a3c1059abe94991"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach Drafts" sheetId="5" r:id="R9661951a316d4734"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6622,7 +6622,7 @@
       <x:c r="P5" s="86"/>
       <x:c r="Q5" s="84"/>
       <x:c r="R5" s="84" t="str">
-        <x:v>Outreach angle: offer independent Web/API VAPT before DewWeb client launches and enterprise security reviews.</x:v>
+        <x:v>Verified public business inbox. Outreach angle: offer independent Web/API VAPT before DewWeb client launches and enterprise security reviews.</x:v>
       </x:c>
       <x:c r="S5" s="1"/>
       <x:c r="T5" s="1"/>
@@ -6653,7 +6653,9 @@
       <x:c r="G6" s="84" t="str">
         <x:v>Founder / Delivery Head</x:v>
       </x:c>
-      <x:c r="H6" s="84"/>
+      <x:c r="H6" s="84" t="str">
+        <x:v>contact@agzenix.com</x:v>
+      </x:c>
       <x:c r="I6" s="84" t="str">
         <x:v>Public company website</x:v>
       </x:c>
@@ -6676,7 +6678,7 @@
       <x:c r="P6" s="86"/>
       <x:c r="Q6" s="84"/>
       <x:c r="R6" s="84" t="str">
-        <x:v>Outreach angle: complement product engineering engagements with independent application-security validation.</x:v>
+        <x:v>Verified public business inbox. Outreach angle: complement product engineering engagements with independent application-security validation.</x:v>
       </x:c>
       <x:c r="S6" s="1"/>
       <x:c r="T6" s="1"/>
@@ -6703,11 +6705,15 @@
       <x:c r="E7" s="84" t="str">
         <x:v>Software development agency</x:v>
       </x:c>
-      <x:c r="F7" s="84"/>
+      <x:c r="F7" s="84" t="str">
+        <x:v>Amol Dhore</x:v>
+      </x:c>
       <x:c r="G7" s="84" t="str">
-        <x:v>Founder / Delivery Head</x:v>
-      </x:c>
-      <x:c r="H7" s="84"/>
+        <x:v>Founder &amp; Director</x:v>
+      </x:c>
+      <x:c r="H7" s="84" t="str">
+        <x:v>admin@tantradev.com</x:v>
+      </x:c>
       <x:c r="I7" s="84" t="str">
         <x:v>Public company website</x:v>
       </x:c>
@@ -6730,7 +6736,7 @@
       <x:c r="P7" s="86"/>
       <x:c r="Q7" s="84"/>
       <x:c r="R7" s="84" t="str">
-        <x:v>Outreach angle: add scoped Web/API VAPT before production launches and for recurring assurance.</x:v>
+        <x:v>Founder identity and public business inbox verified. Outreach angle: add scoped Web/API VAPT before production launches and for recurring assurance.</x:v>
       </x:c>
       <x:c r="S7" s="1"/>
       <x:c r="T7" s="1"/>
@@ -6757,11 +6763,15 @@
       <x:c r="E8" s="84" t="str">
         <x:v>Custom software development</x:v>
       </x:c>
-      <x:c r="F8" s="84"/>
+      <x:c r="F8" s="84" t="str">
+        <x:v>Dharmendra Singh Yadav</x:v>
+      </x:c>
       <x:c r="G8" s="84" t="str">
-        <x:v>Founder / Partnerships Head</x:v>
-      </x:c>
-      <x:c r="H8" s="84"/>
+        <x:v>Founder &amp; Product Engineer</x:v>
+      </x:c>
+      <x:c r="H8" s="84" t="str">
+        <x:v>founder@dharmsy.com</x:v>
+      </x:c>
       <x:c r="I8" s="84" t="str">
         <x:v>Public company website</x:v>
       </x:c>
@@ -6784,7 +6794,7 @@
       <x:c r="P8" s="86"/>
       <x:c r="Q8" s="84"/>
       <x:c r="R8" s="84" t="str">
-        <x:v>Outreach angle: independent security testing for SaaS and API projects delivered to business clients.</x:v>
+        <x:v>Founder identity and public business inbox verified. Outreach angle: independent security testing for SaaS and API projects delivered to business clients.</x:v>
       </x:c>
       <x:c r="S8" s="1"/>
       <x:c r="T8" s="1"/>
@@ -21612,7 +21622,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d99260487c74218"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ab0e82c64714deb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27382,7 +27392,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce700d7b6dc14130"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf7c8aa5de8442a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33304,10 +33314,10 @@
         <x:v>LinkedIn or public business email</x:v>
       </x:c>
       <x:c r="D6" s="22" t="str">
-        <x:v>Hi [Name], I noticed DewWeb Solution works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to offer independent Web/API VAPT before DewWeb client launches and enterprise security reviews. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
+        <x:v>Hello DewWeb Solution team, I noticed DewWeb Solution works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to offer independent Web/API VAPT before DewWeb client launches and enterprise security reviews. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
       </x:c>
       <x:c r="E6" s="22" t="str">
-        <x:v>Hi [Name], following up on my note about independent Web/API VAPT support for DewWeb Solution's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
+        <x:v>Hello DewWeb Solution team, following up on my note about independent Web/API VAPT support for DewWeb Solution's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
       </x:c>
       <x:c r="F6" s="101" t="str">
         <x:v>Needs approval</x:v>
@@ -33344,10 +33354,10 @@
         <x:v>LinkedIn or public business email</x:v>
       </x:c>
       <x:c r="D7" s="22" t="str">
-        <x:v>Hi [Name], I noticed Agzenix works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to complement product engineering engagements with independent application-security validation. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
+        <x:v>Hello Agzenix team, I noticed Agzenix works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to complement product engineering engagements with independent application-security validation. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
       </x:c>
       <x:c r="E7" s="22" t="str">
-        <x:v>Hi [Name], following up on my note about independent Web/API VAPT support for Agzenix's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
+        <x:v>Hello Agzenix team, following up on my note about independent Web/API VAPT support for Agzenix's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
       </x:c>
       <x:c r="F7" s="101" t="str">
         <x:v>Needs approval</x:v>
@@ -33378,16 +33388,16 @@
         <x:v>TantraDev Information Technologies</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>Founder / Delivery Head</x:v>
+        <x:v>Amol Dhore — Founder &amp; Director</x:v>
       </x:c>
       <x:c r="C8" s="22" t="str">
         <x:v>LinkedIn or public business email</x:v>
       </x:c>
       <x:c r="D8" s="22" t="str">
-        <x:v>Hi [Name], I noticed TantraDev Information Technologies works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to add scoped Web/API VAPT before production launches and for recurring assurance. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
+        <x:v>Hi Amol, I noticed TantraDev Information Technologies works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to add scoped Web/API VAPT before production launches and for recurring assurance. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
       </x:c>
       <x:c r="E8" s="22" t="str">
-        <x:v>Hi [Name], following up on my note about independent Web/API VAPT support for TantraDev Information Technologies's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
+        <x:v>Hi Amol, following up on my note about independent Web/API VAPT support for TantraDev Information Technologies's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
       </x:c>
       <x:c r="F8" s="101" t="str">
         <x:v>Needs approval</x:v>
@@ -33418,16 +33428,16 @@
         <x:v>Dharmsy Innovations</x:v>
       </x:c>
       <x:c r="B9" s="22" t="str">
-        <x:v>Founder / Partnerships Head</x:v>
+        <x:v>Dharmendra Singh Yadav — Founder &amp; Product Engineer</x:v>
       </x:c>
       <x:c r="C9" s="22" t="str">
         <x:v>LinkedIn or public business email</x:v>
       </x:c>
       <x:c r="D9" s="22" t="str">
-        <x:v>Hi [Name], I noticed Dharmsy Innovations works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to independent security testing for SaaS and API projects delivered to business clients. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
+        <x:v>Hi Dharmendra, I noticed Dharmsy Innovations works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to independent security testing for SaaS and API projects delivered to business clients. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
       </x:c>
       <x:c r="E9" s="22" t="str">
-        <x:v>Hi [Name], following up on my note about independent Web/API VAPT support for Dharmsy Innovations's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
+        <x:v>Hi Dharmendra, following up on my note about independent Web/API VAPT support for Dharmsy Innovations's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
       </x:c>
       <x:c r="F9" s="101" t="str">
         <x:v>Needs approval</x:v>
@@ -33464,10 +33474,10 @@
         <x:v>LinkedIn or public business email</x:v>
       </x:c>
       <x:c r="D10" s="22" t="str">
-        <x:v>Hi [Name], I noticed Leacotta works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to manual business-logic and access-control testing for multi-tenant SaaS launches. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
+        <x:v>Hello Leacotta team, I noticed Leacotta works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to manual business-logic and access-control testing for multi-tenant SaaS launches. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
       </x:c>
       <x:c r="E10" s="22" t="str">
-        <x:v>Hi [Name], following up on my note about independent Web/API VAPT support for Leacotta's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
+        <x:v>Hello Leacotta team, following up on my note about independent Web/API VAPT support for Leacotta's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
       </x:c>
       <x:c r="F10" s="101" t="str">
         <x:v>Needs approval</x:v>
@@ -33504,10 +33514,10 @@
         <x:v>LinkedIn or public business email</x:v>
       </x:c>
       <x:c r="D11" s="22" t="str">
-        <x:v>Hi [Name], I noticed Vedrisha works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to partner for third-party VAPT evidence on client web and cloud projects. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
+        <x:v>Hello Vedrisha team, I noticed Vedrisha works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to partner for third-party VAPT evidence on client web and cloud projects. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
       </x:c>
       <x:c r="E11" s="22" t="str">
-        <x:v>Hi [Name], following up on my note about independent Web/API VAPT support for Vedrisha's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
+        <x:v>Hello Vedrisha team, following up on my note about independent Web/API VAPT support for Vedrisha's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
       </x:c>
       <x:c r="F11" s="101" t="str">
         <x:v>Needs approval</x:v>
@@ -33544,10 +33554,10 @@
         <x:v>LinkedIn or public business email</x:v>
       </x:c>
       <x:c r="D12" s="22" t="str">
-        <x:v>Hi [Name], I noticed Trimsel works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to independent testing for security-sensitive fintech, healthtech, and SaaS client applications. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
+        <x:v>Hello Trimsel team, I noticed Trimsel works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to independent testing for security-sensitive fintech, healthtech, and SaaS client applications. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
       </x:c>
       <x:c r="E12" s="22" t="str">
-        <x:v>Hi [Name], following up on my note about independent Web/API VAPT support for Trimsel's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
+        <x:v>Hello Trimsel team, following up on my note about independent Web/API VAPT support for Trimsel's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
       </x:c>
       <x:c r="F12" s="101" t="str">
         <x:v>Needs approval</x:v>
@@ -33584,10 +33594,10 @@
         <x:v>LinkedIn or public business email</x:v>
       </x:c>
       <x:c r="D13" s="22" t="str">
-        <x:v>Hi [Name], I noticed Hexolve works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to offer pre-launch Web/API VAPT as an independent quality gate for client products. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
+        <x:v>Hello Hexolve team, I noticed Hexolve works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to offer pre-launch Web/API VAPT as an independent quality gate for client products. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
       </x:c>
       <x:c r="E13" s="22" t="str">
-        <x:v>Hi [Name], following up on my note about independent Web/API VAPT support for Hexolve's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
+        <x:v>Hello Hexolve team, following up on my note about independent Web/API VAPT support for Hexolve's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
       </x:c>
       <x:c r="F13" s="101" t="str">
         <x:v>Needs approval</x:v>
@@ -33624,10 +33634,10 @@
         <x:v>LinkedIn or public business email</x:v>
       </x:c>
       <x:c r="D14" s="22" t="str">
-        <x:v>Hi [Name], I noticed Bytes Brothers works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to test tenant isolation, authentication, authorization, billing, and API integrations before handover. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
+        <x:v>Hello Bytes Brothers team, I noticed Bytes Brothers works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to test tenant isolation, authentication, authorization, billing, and API integrations before handover. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
       </x:c>
       <x:c r="E14" s="22" t="str">
-        <x:v>Hi [Name], following up on my note about independent Web/API VAPT support for Bytes Brothers's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
+        <x:v>Hello Bytes Brothers team, following up on my note about independent Web/API VAPT support for Bytes Brothers's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
       </x:c>
       <x:c r="F14" s="101" t="str">
         <x:v>Needs approval</x:v>
@@ -33664,10 +33674,10 @@
         <x:v>LinkedIn or public business email</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
-        <x:v>Hi [Name], I noticed ThreeAtoms works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to scoped application testing for startup and enterprise web projects before release. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
+        <x:v>Hello ThreeAtoms team, I noticed ThreeAtoms works on SaaS and web-software projects. I run CyberVSI, providing independent web application and API penetration testing. We are exploring partnerships with development teams that need a security-testing partner before client launches or security reviews. A relevant fit may be to scoped application testing for startup and enterprise web projects before release. Would you be open to a short discussion? I can share our testing process and sanitized sample report.</x:v>
       </x:c>
       <x:c r="E15" s="23" t="str">
-        <x:v>Hi [Name], following up on my note about independent Web/API VAPT support for ThreeAtoms's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
+        <x:v>Hello ThreeAtoms team, following up on my note about independent Web/API VAPT support for ThreeAtoms's client projects. If an upcoming release or customer review needs third-party testing, I can share a sample deliverable and propose a clearly bounded scope. Would that be useful?</x:v>
       </x:c>
       <x:c r="F15" s="102" t="str">
         <x:v>Needs approval</x:v>

</xml_diff>